<commit_message>
Improve article interaction tracking and SEO features. Enhanced user interaction tracking in article-renderer.js and updated HTML templates to include structured data for better SEO. Adjusted navigation links and mailto functionality for improved user experience.
</commit_message>
<xml_diff>
--- a/framework.xlsx
+++ b/framework.xlsx
@@ -1518,7 +1518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2174,17 +2174,17 @@
       </c>
       <c r="B19" s="11" t="inlineStr">
         <is>
-          <t>インタビューカード3件</t>
+          <t>取材協力者のリアルな声（インタビュー）</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>利用者の生の声をQ&amp;A形式で掲載</t>
+          <t>第三者性と納得感の補強（Q&amp;A＋観察メモ）</t>
         </is>
       </c>
       <c r="D19" s="11" t="inlineStr">
         <is>
-          <t>氏名・年齢・性別 / 質問 / 回答 / 記者観察</t>
+          <t>interviews[] の内容をカード化（結果バッジ＋Q&amp;A＋obs）</t>
         </is>
       </c>
       <c r="E19" s="11" t="inlineStr">
@@ -2194,12 +2194,12 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>reviews[].name / .age / .text</t>
+          <t>interviews[].name / bg / resultType / resultLabel / qa[].q / qa[].a / obs</t>
         </is>
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Q&amp;A形式 / 記者観察メモ付き</t>
+          <t>resultType（success/other）でバッジ色を切替</t>
         </is>
       </c>
     </row>
@@ -2322,17 +2322,17 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>最終評決</t>
+          <t>最終評決（記者総評）</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>記者の総評</t>
+          <t>全体の論点をまとめ意思決定を支援</t>
         </is>
       </c>
       <c r="D23" s="11" t="inlineStr">
         <is>
-          <t>まとめコメント</t>
+          <t>cuttingSummary の label/text を強調枠で提示</t>
         </is>
       </c>
       <c r="E23" s="11" t="inlineStr">
@@ -2342,12 +2342,12 @@
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>storyText[]</t>
+          <t>cuttingSummary.label / cuttingSummary.text</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>強調枠</t>
+          <t>記事の締め・判断材料の要約</t>
         </is>
       </c>
     </row>
@@ -2570,6 +2570,117 @@
       <c r="G29" s="11" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>STORY</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>このメディアを始めた理由</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>ブランド/姿勢の納得感を作る</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>storyImg + storyText[]（段落）</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>.story-section</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>.story-content / .story-img / blockquote</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>記事の背景・理念を段落で提示</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SEO/STRUCTURED DATA</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>OGP/メタタグ（JSで上書き）</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>シェア/検索スニペット最適化</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>document.title + meta description + og:* + og:image</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>(metaタグ)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>title / metaDesc / ogImage</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>article-renderer.js の setMeta / ogImageAbsolute</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>SEO/STRUCTURED DATA</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>JSON-LD（Article/Breadcrumb/FAQ）</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Google/AIによる記事理解補助</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Article / BreadcrumbList / FAQPage（最大10問）</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>&lt;script type="application/ld+json"&gt;</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>jsonld-breadcrumb / jsonld-article / jsonld-faq</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>article-renderer.js の upsertJSONLD</t>
         </is>
       </c>
     </row>

</xml_diff>